<commit_message>
docs(tutorials): the reinforce sheets show what their formulas answer
Dir/Appl formula cells carry cached values (XML surgery, formulas
untouched, loader asserted identical) so renders and non-Excel readers
see what Excel shows; both sheet renders regenerated. LEM-8's intro
names the base 10 ft below the slope (not in the drawing) and the
profile step includes Max Depth in the entry instruction.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_reinforce.xlsx
+++ b/docs/lem/files/xslope_reinforce.xlsx
@@ -1907,13 +1907,13 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="3" t="str">
         <f>IF($G3="","",IFERROR(VLOOKUP($G3,$Z$8:$AB$11,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="I3" s="3">
+        <v>Tangent</v>
+      </c>
+      <c r="I3" s="3" t="str">
         <f>IF($G3="","",IFERROR(VLOOKUP($G3,$Z$8:$AB$11,3,0),""))</f>
-        <v/>
+        <v>Active</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>800</v>
@@ -1980,13 +1980,13 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="3" t="str">
         <f>IF($G4="","",IFERROR(VLOOKUP($G4,$Z$8:$AB$11,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="I4" s="3">
+        <v>Tangent</v>
+      </c>
+      <c r="I4" s="3" t="str">
         <f>IF($G4="","",IFERROR(VLOOKUP($G4,$Z$8:$AB$11,3,0),""))</f>
-        <v/>
+        <v>Active</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>800</v>
@@ -2043,13 +2043,13 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="3" t="str">
         <f>IF($G5="","",IFERROR(VLOOKUP($G5,$Z$8:$AB$11,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="I5" s="3">
+        <v>Tangent</v>
+      </c>
+      <c r="I5" s="3" t="str">
         <f>IF($G5="","",IFERROR(VLOOKUP($G5,$Z$8:$AB$11,3,0),""))</f>
-        <v/>
+        <v>Active</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>800</v>
@@ -2106,13 +2106,13 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="3" t="str">
         <f>IF($G6="","",IFERROR(VLOOKUP($G6,$Z$8:$AB$11,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="I6" s="3">
+        <v>Tangent</v>
+      </c>
+      <c r="I6" s="3" t="str">
         <f>IF($G6="","",IFERROR(VLOOKUP($G6,$Z$8:$AB$11,3,0),""))</f>
-        <v/>
+        <v>Active</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>800</v>
@@ -2164,13 +2164,13 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="3" t="str">
         <f>IF($G7="","",IFERROR(VLOOKUP($G7,$Z$8:$AB$11,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="I7" s="3">
+        <v>Tangent</v>
+      </c>
+      <c r="I7" s="3" t="str">
         <f>IF($G7="","",IFERROR(VLOOKUP($G7,$Z$8:$AB$11,3,0),""))</f>
-        <v/>
+        <v>Active</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>800</v>
@@ -2222,13 +2222,13 @@
           <t>Geosynthetic</t>
         </is>
       </c>
-      <c r="H8" s="3">
+      <c r="H8" s="3" t="str">
         <f>IF($G8="","",IFERROR(VLOOKUP($G8,$Z$8:$AB$11,2,0),""))</f>
-        <v/>
-      </c>
-      <c r="I8" s="3">
+        <v>Tangent</v>
+      </c>
+      <c r="I8" s="3" t="str">
         <f>IF($G8="","",IFERROR(VLOOKUP($G8,$Z$8:$AB$11,3,0),""))</f>
-        <v/>
+        <v>Active</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>800</v>

</xml_diff>

<commit_message>
docs(lem): the geogrid sample's Tres cells go blank
FEM-only residual capacity the LEM sample never chose — blank reads as
unspecified. Formulas untouched, Spencer search 1.5867 unchanged,
render regenerated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_reinforce.xlsx
+++ b/docs/lem/files/xslope_reinforce.xlsx
@@ -1933,9 +1933,7 @@
       <c r="O3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="P3" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="P3" s="3"/>
       <c r="Q3" s="3" t="n"/>
       <c r="R3" s="3" t="n"/>
       <c r="Z3" t="inlineStr">
@@ -2006,9 +2004,7 @@
       <c r="O4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="P4" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="P4" s="3"/>
       <c r="Q4" s="3" t="n"/>
       <c r="R4" s="3" t="n"/>
       <c r="Z4" t="inlineStr">
@@ -2069,9 +2065,7 @@
       <c r="O5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="P5" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="P5" s="3"/>
       <c r="Q5" s="3" t="n"/>
       <c r="R5" s="3" t="n"/>
       <c r="Z5" t="inlineStr">
@@ -2132,9 +2126,7 @@
       <c r="O6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="P6" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="P6" s="3"/>
       <c r="Q6" s="3" t="n"/>
       <c r="R6" s="3" t="n"/>
     </row>
@@ -2190,9 +2182,7 @@
       <c r="O7" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="P7" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="P7" s="3"/>
       <c r="Q7" s="3" t="n"/>
       <c r="R7" s="3" t="n"/>
     </row>
@@ -2248,9 +2238,7 @@
       <c r="O8" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="P8" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="P8" s="3"/>
       <c r="Q8" s="3" t="n"/>
       <c r="R8" s="3" t="n"/>
       <c r="Z8" t="inlineStr">

</xml_diff>